<commit_message>
feat(schema): support scoped config outputs
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Economy.xlsx
+++ b/examples/showcase/data/Economy.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="457">
   <si>
     <t>@table</t>
   </si>
@@ -41,10 +41,16 @@
     <t>id</t>
   </si>
   <si>
+    <t>@scope</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
     <t>@schema</t>
   </si>
   <si>
-    <t>fb9f9a6efc928f54</t>
+    <t>d73be5f5f0b43620</t>
   </si>
   <si>
     <t>#name</t>
@@ -71,6 +77,9 @@
     <t>enum&lt;ResourceKind&gt;</t>
   </si>
   <si>
+    <t>#scope</t>
+  </si>
+  <si>
     <t>#rule</t>
   </si>
   <si>
@@ -125,7 +134,7 @@
     <t>list</t>
   </si>
   <si>
-    <t>1121be035e2d102d</t>
+    <t>29a78037800e1f0d</t>
   </si>
   <si>
     <t>shop_id</t>
@@ -374,7 +383,7 @@
     <t>Recipe</t>
   </si>
   <si>
-    <t>c7d7333d6fa37cec</t>
+    <t>8db60b21001cd79c</t>
   </si>
   <si>
     <t>result_item</t>
@@ -602,7 +611,7 @@
     <t>GachaPool</t>
   </si>
   <si>
-    <t>cfa9227062e6c47e</t>
+    <t>c8754f01535034ea</t>
   </si>
   <si>
     <t>cost</t>
@@ -638,7 +647,7 @@
     <t>GachaItem</t>
   </si>
   <si>
-    <t>0fbc411230fbb853</t>
+    <t>a5ceab1ecef1335f</t>
   </si>
   <si>
     <t>pool_id</t>
@@ -797,7 +806,7 @@
     <t>EquipmentSet</t>
   </si>
   <si>
-    <t>6469050bb5882ec0</t>
+    <t>8e8278844e0723f8</t>
   </si>
   <si>
     <t>item_ids</t>
@@ -935,7 +944,7 @@
     <t>Achievement</t>
   </si>
   <si>
-    <t>77dbe69eed12ff37</t>
+    <t>6ee1fabd128867ef</t>
   </si>
   <si>
     <t>title_key</t>
@@ -1316,7 +1325,7 @@
     <t>level</t>
   </si>
   <si>
-    <t>0db99fa9ff187953</t>
+    <t>fa7d329b8bf6b387</t>
   </si>
   <si>
     <t>perks</t>
@@ -1714,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1749,120 +1758,142 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B5" t="s">
         <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>21</v>
       </c>
-      <c r="C11" t="s">
-        <v>22</v>
+      <c r="D11" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
         <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
         <v>31</v>
       </c>
-      <c r="C15" t="s">
-        <v>22</v>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1872,7 +1903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1880,7 +1911,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1888,7 +1919,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1901,241 +1932,238 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B5" t="s">
         <v>37</v>
-      </c>
-      <c r="E6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
         <v>40</v>
       </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>41</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>42</v>
-      </c>
-      <c r="F8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
         <v>47</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" t="s">
-        <v>62</v>
-      </c>
-      <c r="D16" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="E18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
-      </c>
-      <c r="E19" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2143,13 +2171,16 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D21" t="s">
-        <v>48</v>
+        <v>75</v>
+      </c>
+      <c r="E21" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2157,134 +2188,131 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
         <v>77</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
-      </c>
-      <c r="E23" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B25" t="s">
         <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D25" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="E25" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" t="s">
         <v>61</v>
-      </c>
-      <c r="C26" t="s">
-        <v>81</v>
-      </c>
-      <c r="D26" t="s">
-        <v>63</v>
-      </c>
-      <c r="E26" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="E28" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D29" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D30" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -2292,13 +2320,16 @@
         <v>26</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="C31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D31" t="s">
-        <v>48</v>
+        <v>75</v>
+      </c>
+      <c r="E31" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2306,432 +2337,460 @@
         <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="C32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D32" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D33" t="s">
-        <v>54</v>
-      </c>
-      <c r="E33" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B34" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C34" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B35" t="s">
         <v>55</v>
       </c>
       <c r="C35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D35" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="E35" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B36" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" t="s">
+        <v>92</v>
+      </c>
+      <c r="D36" t="s">
         <v>61</v>
-      </c>
-      <c r="C36" t="s">
-        <v>91</v>
-      </c>
-      <c r="D36" t="s">
-        <v>63</v>
-      </c>
-      <c r="E36" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D37" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B38" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C38" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D38" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="E38" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C39" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D39" t="s">
-        <v>72</v>
-      </c>
-      <c r="E39" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B40" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C40" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D41" t="s">
-        <v>48</v>
+        <v>75</v>
+      </c>
+      <c r="E41" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B42" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="C42" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D42" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B43" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D43" t="s">
-        <v>54</v>
-      </c>
-      <c r="E43" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C44" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D44" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B45" t="s">
         <v>55</v>
       </c>
       <c r="C45" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D45" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="E45" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C46" t="s">
+        <v>102</v>
+      </c>
+      <c r="D46" t="s">
         <v>61</v>
-      </c>
-      <c r="C46" t="s">
-        <v>101</v>
-      </c>
-      <c r="D46" t="s">
-        <v>63</v>
-      </c>
-      <c r="E46" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B47" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C47" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D47" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B48" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D48" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="E48" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C49" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D49" t="s">
-        <v>72</v>
-      </c>
-      <c r="E49" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C50" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D50" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B51" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D51" t="s">
-        <v>48</v>
+        <v>75</v>
+      </c>
+      <c r="E51" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B52" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="C52" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D52" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B53" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C53" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D53" t="s">
-        <v>54</v>
-      </c>
-      <c r="E53" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B54" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D54" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B55" t="s">
         <v>55</v>
       </c>
       <c r="C55" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D55" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="E55" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B56" t="s">
+        <v>59</v>
+      </c>
+      <c r="C56" t="s">
+        <v>112</v>
+      </c>
+      <c r="D56" t="s">
         <v>61</v>
-      </c>
-      <c r="C56" t="s">
-        <v>111</v>
-      </c>
-      <c r="D56" t="s">
-        <v>63</v>
-      </c>
-      <c r="E56" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B57" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C57" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D57" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B58" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D58" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="E58" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B59" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C59" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D59" t="s">
-        <v>72</v>
-      </c>
-      <c r="E59" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B60" t="s">
+        <v>70</v>
+      </c>
+      <c r="C60" t="s">
+        <v>116</v>
+      </c>
+      <c r="D60" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>33</v>
+      </c>
+      <c r="B61" t="s">
         <v>73</v>
       </c>
-      <c r="C60" t="s">
-        <v>115</v>
-      </c>
-      <c r="D60" t="s">
+      <c r="C61" t="s">
+        <v>117</v>
+      </c>
+      <c r="D61" t="s">
         <v>75</v>
+      </c>
+      <c r="E61" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>33</v>
+      </c>
+      <c r="B62" t="s">
+        <v>76</v>
+      </c>
+      <c r="C62" t="s">
+        <v>118</v>
+      </c>
+      <c r="D62" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2741,7 +2800,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2749,7 +2808,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2773,398 +2832,420 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D6" t="s">
-        <v>119</v>
+      <c r="B5" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>121</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>123</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>125</v>
-      </c>
-      <c r="B12" t="s">
-        <v>126</v>
-      </c>
-      <c r="C12" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C13" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C14" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B15" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C15" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B17" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C17" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B18" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C18" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B19" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C19" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B20" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C20" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="C21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" t="s">
         <v>154</v>
-      </c>
-      <c r="B22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
         <v>156</v>
-      </c>
-      <c r="B23" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>157</v>
+      </c>
+      <c r="B24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" t="s">
         <v>158</v>
-      </c>
-      <c r="B24" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" t="s">
         <v>160</v>
-      </c>
-      <c r="B25" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>161</v>
+      </c>
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" t="s">
         <v>162</v>
-      </c>
-      <c r="B26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C26" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
+        <v>163</v>
+      </c>
+      <c r="B27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" t="s">
         <v>164</v>
-      </c>
-      <c r="B27" t="s">
-        <v>65</v>
-      </c>
-      <c r="C27" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
+        <v>165</v>
+      </c>
+      <c r="B28" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" t="s">
         <v>166</v>
-      </c>
-      <c r="B28" t="s">
-        <v>68</v>
-      </c>
-      <c r="C28" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
+        <v>167</v>
+      </c>
+      <c r="B29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" t="s">
         <v>168</v>
-      </c>
-      <c r="B29" t="s">
-        <v>71</v>
-      </c>
-      <c r="C29" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
+        <v>169</v>
+      </c>
+      <c r="B30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" t="s">
         <v>170</v>
-      </c>
-      <c r="B30" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>171</v>
+      </c>
+      <c r="B31" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" t="s">
         <v>172</v>
-      </c>
-      <c r="B31" t="s">
-        <v>76</v>
-      </c>
-      <c r="C31" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B32" t="s">
         <v>77</v>
       </c>
       <c r="C32" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
+        <v>175</v>
+      </c>
+      <c r="B33" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" t="s">
         <v>176</v>
-      </c>
-      <c r="B33" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
+        <v>177</v>
+      </c>
+      <c r="B34" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" t="s">
         <v>178</v>
-      </c>
-      <c r="B34" t="s">
-        <v>79</v>
-      </c>
-      <c r="C34" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
+        <v>179</v>
+      </c>
+      <c r="B35" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" t="s">
         <v>180</v>
-      </c>
-      <c r="B35" t="s">
-        <v>80</v>
-      </c>
-      <c r="C35" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
+        <v>181</v>
+      </c>
+      <c r="B36" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" t="s">
         <v>182</v>
-      </c>
-      <c r="B36" t="s">
-        <v>81</v>
-      </c>
-      <c r="C36" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
+        <v>183</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" t="s">
         <v>184</v>
-      </c>
-      <c r="B37" t="s">
-        <v>82</v>
-      </c>
-      <c r="C37" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>185</v>
+      </c>
+      <c r="B38" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" t="s">
         <v>186</v>
-      </c>
-      <c r="B38" t="s">
-        <v>83</v>
-      </c>
-      <c r="C38" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>187</v>
+      </c>
+      <c r="B39" t="s">
+        <v>85</v>
+      </c>
+      <c r="C39" t="s">
         <v>188</v>
-      </c>
-      <c r="B39" t="s">
-        <v>84</v>
-      </c>
-      <c r="C39" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>189</v>
+      </c>
+      <c r="B40" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" t="s">
         <v>190</v>
       </c>
-      <c r="B40" t="s">
-        <v>85</v>
-      </c>
-      <c r="C40" t="s">
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
         <v>191</v>
+      </c>
+      <c r="B41" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -3174,7 +3255,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3182,7 +3263,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3206,101 +3287,123 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>194</v>
+      <c r="B5" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>195</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>196</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>197</v>
+        <v>21</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>198</v>
-      </c>
-      <c r="B12" t="s">
-        <v>199</v>
-      </c>
-      <c r="C12" t="s">
-        <v>200</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
+        <v>198</v>
+      </c>
+      <c r="B13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C13" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
         <v>201</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>202</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C14" t="s">
         <v>203</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>204</v>
+      </c>
+      <c r="B15" t="s">
+        <v>205</v>
+      </c>
+      <c r="C15" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -3310,7 +3413,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3318,7 +3421,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3326,7 +3429,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3339,52 +3442,43 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>206</v>
-      </c>
-      <c r="C6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" t="s">
-        <v>207</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="B5" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>209</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
         <v>210</v>
@@ -3395,77 +3489,83 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>212</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>213</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>195</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>212</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>195</v>
-      </c>
-      <c r="B12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" t="s">
-        <v>213</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D14" t="s">
         <v>55</v>
@@ -3473,139 +3573,139 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C16" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D16" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C20" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D20" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C21" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D21" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B22" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C22" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C23" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C24" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D24" t="s">
         <v>55</v>
@@ -3613,86 +3713,86 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C25" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D26" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C27" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D27" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C28" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B29" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D29" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D30" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -3700,13 +3800,13 @@
         <v>198</v>
       </c>
       <c r="B31" t="s">
-        <v>217</v>
+        <v>107</v>
       </c>
       <c r="C31" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D31" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -3714,38 +3814,38 @@
         <v>198</v>
       </c>
       <c r="B32" t="s">
-        <v>218</v>
+        <v>108</v>
       </c>
       <c r="C32" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D32" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D33" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C34" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D34" t="s">
         <v>55</v>
@@ -3753,139 +3853,139 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B35" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D35" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B36" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C36" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D36" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B37" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C37" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D37" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B38" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C38" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D38" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B39" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C39" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D39" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B40" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D40" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B41" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C41" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B42" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C42" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D42" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B43" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C43" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D43" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B44" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C44" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D44" t="s">
         <v>55</v>
@@ -3893,86 +3993,86 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B45" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C45" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D45" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B46" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C46" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D46" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B47" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C47" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D47" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B48" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C48" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D48" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B49" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C49" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D49" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B50" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C50" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D50" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3980,13 +4080,13 @@
         <v>201</v>
       </c>
       <c r="B51" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C51" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D51" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3994,38 +4094,38 @@
         <v>201</v>
       </c>
       <c r="B52" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C52" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D52" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B53" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C53" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D53" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B54" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C54" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D54" t="s">
         <v>55</v>
@@ -4033,139 +4133,139 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B55" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C55" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D55" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B56" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C56" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D56" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B57" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C57" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D57" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B58" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C58" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D58" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B59" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C59" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D59" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B60" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C60" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D60" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B61" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C61" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D61" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B62" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C62" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D62" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B63" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C63" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D63" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B64" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C64" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D64" t="s">
         <v>55</v>
@@ -4173,86 +4273,114 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B65" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C65" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D65" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B66" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C66" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D66" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B67" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C67" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D67" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B68" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C68" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D68" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B69" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C69" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D69" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B70" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C70" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D70" t="s">
-        <v>46</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" t="s">
+        <v>204</v>
+      </c>
+      <c r="B71" t="s">
+        <v>258</v>
+      </c>
+      <c r="C71" t="s">
+        <v>218</v>
+      </c>
+      <c r="D71" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" t="s">
+        <v>204</v>
+      </c>
+      <c r="B72" t="s">
+        <v>259</v>
+      </c>
+      <c r="C72" t="s">
+        <v>219</v>
+      </c>
+      <c r="D72" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -4262,7 +4390,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4270,7 +4398,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -4294,220 +4422,245 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>259</v>
-      </c>
-      <c r="E6" t="s">
-        <v>260</v>
+      <c r="B5" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E7" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>264</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>263</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>264</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>265</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>266</v>
+        <v>124</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>267</v>
-      </c>
-      <c r="B12" t="s">
-        <v>268</v>
-      </c>
-      <c r="C12" t="s">
-        <v>269</v>
-      </c>
-      <c r="D12" t="s">
-        <v>270</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B13" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C13" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D13" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B14" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C14" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D14" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="B15" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="C15" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="D15" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B16" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C16" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D16" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B17" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="C17" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="D17" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B18" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="C18" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D18" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B19" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="C19" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="D19" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
+        <v>294</v>
+      </c>
+      <c r="B20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C20" t="s">
+        <v>296</v>
+      </c>
+      <c r="D20" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>298</v>
+      </c>
+      <c r="B21" t="s">
         <v>299</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C21" t="s">
         <v>300</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D21" t="s">
         <v>301</v>
       </c>
-      <c r="D20" t="s">
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
         <v>302</v>
+      </c>
+      <c r="B22" t="s">
+        <v>303</v>
+      </c>
+      <c r="C22" t="s">
+        <v>304</v>
+      </c>
+      <c r="D22" t="s">
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -4517,7 +4670,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4525,7 +4678,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -4549,500 +4702,525 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>305</v>
-      </c>
-      <c r="D6" t="s">
-        <v>306</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="B5" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D7" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E7" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>308</v>
       </c>
       <c r="D8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>311</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>309</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>310</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>311</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>312</v>
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>313</v>
-      </c>
-      <c r="B12" t="s">
-        <v>314</v>
-      </c>
-      <c r="C12" t="s">
-        <v>315</v>
-      </c>
-      <c r="D12" t="s">
-        <v>316</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="B13" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C13" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="D13" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="B14" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="C14" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="D14" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B15" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="C15" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="D15" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B16" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="C16" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="D16" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B17" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="C17" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="D17" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="B18" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="C18" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D18" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="B19" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C19" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D19" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B20" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="C20" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="D20" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="B21" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="C21" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D21" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B22" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="C22" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D22" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B23" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="C23" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="D23" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="B24" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="C24" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="D24" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B25" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="C25" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="D25" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B26" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="C26" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="D26" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="B27" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="C27" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="D27" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B28" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C28" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D28" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B29" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C29" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="D29" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B30" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C30" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="D30" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B31" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="C31" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="D31" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="B32" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="C32" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="D32" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="B33" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="C33" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="D33" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="B34" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="C34" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="D34" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="B35" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C35" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="D35" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="B36" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="C36" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="D36" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="B37" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="C37" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="D37" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="B38" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="C38" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="D38" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="B39" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="C39" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="D39" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
+        <v>420</v>
+      </c>
+      <c r="B40" t="s">
+        <v>421</v>
+      </c>
+      <c r="C40" t="s">
+        <v>422</v>
+      </c>
+      <c r="D40" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>424</v>
+      </c>
+      <c r="B41" t="s">
         <v>425</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C41" t="s">
         <v>426</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D41" t="s">
         <v>427</v>
       </c>
-      <c r="D40" t="s">
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
         <v>428</v>
+      </c>
+      <c r="B42" t="s">
+        <v>429</v>
+      </c>
+      <c r="C42" t="s">
+        <v>430</v>
+      </c>
+      <c r="D42" t="s">
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -5052,7 +5230,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -5060,7 +5238,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -5076,7 +5254,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -5084,112 +5262,112 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
-        <v>430</v>
-      </c>
-      <c r="C6" t="s">
-        <v>194</v>
-      </c>
-      <c r="D6" t="s">
-        <v>432</v>
+      <c r="B5" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="C7" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>433</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>197</v>
       </c>
       <c r="D8" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>436</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>434</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>435</v>
+        <v>47</v>
+      </c>
+      <c r="D11" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" t="s">
-        <v>436</v>
-      </c>
-      <c r="C12" t="s">
-        <v>437</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
+        <v>437</v>
+      </c>
+      <c r="C13" t="s">
         <v>438</v>
-      </c>
-      <c r="C13" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
+        <v>439</v>
+      </c>
+      <c r="C14" t="s">
         <v>440</v>
-      </c>
-      <c r="C14" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -5197,65 +5375,87 @@
         <v>55</v>
       </c>
       <c r="B15" t="s">
+        <v>441</v>
+      </c>
+      <c r="C15" t="s">
         <v>442</v>
-      </c>
-      <c r="C15" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B16" t="s">
+        <v>443</v>
+      </c>
+      <c r="C16" t="s">
         <v>444</v>
-      </c>
-      <c r="C16" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
+        <v>445</v>
+      </c>
+      <c r="C17" t="s">
         <v>446</v>
-      </c>
-      <c r="C17" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
+        <v>447</v>
+      </c>
+      <c r="C18" t="s">
         <v>448</v>
-      </c>
-      <c r="C18" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
+        <v>449</v>
+      </c>
+      <c r="C19" t="s">
         <v>450</v>
-      </c>
-      <c r="C19" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>451</v>
+      </c>
+      <c r="C20" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
         <v>73</v>
       </c>
-      <c r="B20" t="s">
-        <v>452</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="B21" t="s">
         <v>453</v>
+      </c>
+      <c r="C21" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" t="s">
+        <v>455</v>
+      </c>
+      <c r="C22" t="s">
+        <v>456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(input): add tuple list parser
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Economy.xlsx
+++ b/examples/showcase/data/Economy.xlsx
@@ -383,7 +383,7 @@
     <t>Recipe</t>
   </si>
   <si>
-    <t>e5fe72682634ed92</t>
+    <t>62064f06c1c0c079</t>
   </si>
   <si>
     <t>result_item</t>
@@ -392,10 +392,10 @@
     <t>materials</t>
   </si>
   <si>
-    <t>list&lt;struct&lt;ResourceCost&gt;&gt;</t>
-  </si>
-  <si>
-    <t>required;parser=json</t>
+    <t>list&lt;struct&lt;ResourceCost&gt;&gt;(kind: enum&lt;ResourceKind&gt;, id: i32, count: i32)</t>
+  </si>
+  <si>
+    <t>required;parser=tuple_list</t>
   </si>
   <si>
     <t>11001</t>
@@ -404,7 +404,7 @@
     <t>1004</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1005,"count":3 },{"kind":"Gold","id":0,"count":110 }]</t>
+    <t>Item,1005,3|Gold,0,110</t>
   </si>
   <si>
     <t>11002</t>
@@ -413,7 +413,7 @@
     <t>1005</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1006,"count":4 },{"kind":"Gold","id":0,"count":120 }]</t>
+    <t>Item,1006,4|Gold,0,120</t>
   </si>
   <si>
     <t>11003</t>
@@ -422,7 +422,7 @@
     <t>1006</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1007,"count":5 },{"kind":"Gold","id":0,"count":130 }]</t>
+    <t>Item,1007,5|Gold,0,130</t>
   </si>
   <si>
     <t>11004</t>
@@ -431,7 +431,7 @@
     <t>1007</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1008,"count":2 },{"kind":"Gold","id":0,"count":140 }]</t>
+    <t>Item,1008,2|Gold,0,140</t>
   </si>
   <si>
     <t>11005</t>
@@ -440,7 +440,7 @@
     <t>1008</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1009,"count":3 },{"kind":"Gold","id":0,"count":150 }]</t>
+    <t>Item,1009,3|Gold,0,150</t>
   </si>
   <si>
     <t>11006</t>
@@ -449,7 +449,7 @@
     <t>1009</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1010,"count":4 },{"kind":"Gold","id":0,"count":160 }]</t>
+    <t>Item,1010,4|Gold,0,160</t>
   </si>
   <si>
     <t>11007</t>
@@ -458,7 +458,7 @@
     <t>1010</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1011,"count":5 },{"kind":"Gold","id":0,"count":170 }]</t>
+    <t>Item,1011,5|Gold,0,170</t>
   </si>
   <si>
     <t>11008</t>
@@ -467,7 +467,7 @@
     <t>1011</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1012,"count":2 },{"kind":"Gold","id":0,"count":180 }]</t>
+    <t>Item,1012,2|Gold,0,180</t>
   </si>
   <si>
     <t>11009</t>
@@ -476,7 +476,7 @@
     <t>1012</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1013,"count":3 },{"kind":"Gold","id":0,"count":190 }]</t>
+    <t>Item,1013,3|Gold,0,190</t>
   </si>
   <si>
     <t>11010</t>
@@ -485,127 +485,127 @@
     <t>1013</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1014,"count":4 },{"kind":"Gold","id":0,"count":200 }]</t>
+    <t>Item,1014,4|Gold,0,200</t>
   </si>
   <si>
     <t>11011</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1015,"count":5 },{"kind":"Gold","id":0,"count":210 }]</t>
+    <t>Item,1015,5|Gold,0,210</t>
   </si>
   <si>
     <t>11012</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1016,"count":2 },{"kind":"Gold","id":0,"count":220 }]</t>
+    <t>Item,1016,2|Gold,0,220</t>
   </si>
   <si>
     <t>11013</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1017,"count":3 },{"kind":"Gold","id":0,"count":230 }]</t>
+    <t>Item,1017,3|Gold,0,230</t>
   </si>
   <si>
     <t>11014</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1018,"count":4 },{"kind":"Gold","id":0,"count":240 }]</t>
+    <t>Item,1018,4|Gold,0,240</t>
   </si>
   <si>
     <t>11015</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1019,"count":5 },{"kind":"Gold","id":0,"count":250 }]</t>
+    <t>Item,1019,5|Gold,0,250</t>
   </si>
   <si>
     <t>11016</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1020,"count":2 },{"kind":"Gold","id":0,"count":260 }]</t>
+    <t>Item,1020,2|Gold,0,260</t>
   </si>
   <si>
     <t>11017</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1021,"count":3 },{"kind":"Gold","id":0,"count":270 }]</t>
+    <t>Item,1021,3|Gold,0,270</t>
   </si>
   <si>
     <t>11018</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1022,"count":4 },{"kind":"Gold","id":0,"count":280 }]</t>
+    <t>Item,1022,4|Gold,0,280</t>
   </si>
   <si>
     <t>11019</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1023,"count":5 },{"kind":"Gold","id":0,"count":290 }]</t>
+    <t>Item,1023,5|Gold,0,290</t>
   </si>
   <si>
     <t>11020</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1024,"count":2 },{"kind":"Gold","id":0,"count":300 }]</t>
+    <t>Item,1024,2|Gold,0,300</t>
   </si>
   <si>
     <t>11021</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1025,"count":3 },{"kind":"Gold","id":0,"count":310 }]</t>
+    <t>Item,1025,3|Gold,0,310</t>
   </si>
   <si>
     <t>11022</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1026,"count":4 },{"kind":"Gold","id":0,"count":320 }]</t>
+    <t>Item,1026,4|Gold,0,320</t>
   </si>
   <si>
     <t>11023</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1027,"count":5 },{"kind":"Gold","id":0,"count":330 }]</t>
+    <t>Item,1027,5|Gold,0,330</t>
   </si>
   <si>
     <t>11024</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1028,"count":2 },{"kind":"Gold","id":0,"count":340 }]</t>
+    <t>Item,1028,2|Gold,0,340</t>
   </si>
   <si>
     <t>11025</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1029,"count":3 },{"kind":"Gold","id":0,"count":350 }]</t>
+    <t>Item,1029,3|Gold,0,350</t>
   </si>
   <si>
     <t>11026</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1030,"count":4 },{"kind":"Gold","id":0,"count":360 }]</t>
+    <t>Item,1030,4|Gold,0,360</t>
   </si>
   <si>
     <t>11027</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1031,"count":5 },{"kind":"Gold","id":0,"count":370 }]</t>
+    <t>Item,1031,5|Gold,0,370</t>
   </si>
   <si>
     <t>11028</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1032,"count":2 },{"kind":"Gold","id":0,"count":380 }]</t>
+    <t>Item,1032,2|Gold,0,380</t>
   </si>
   <si>
     <t>11029</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1033,"count":3 },{"kind":"Gold","id":0,"count":390 }]</t>
+    <t>Item,1033,3|Gold,0,390</t>
   </si>
   <si>
     <t>11030</t>
   </si>
   <si>
-    <t>[{"kind":"Item","id":1034,"count":4 },{"kind":"Gold","id":0,"count":400 }]</t>
+    <t>Item,1034,4|Gold,0,400</t>
   </si>
   <si>
     <t>GachaPool</t>

</xml_diff>

<commit_message>
fix(excel): align template data rows with field headers
</commit_message>
<xml_diff>
--- a/examples/showcase/data/Economy.xlsx
+++ b/examples/showcase/data/Economy.xlsx
@@ -2138,57 +2138,57 @@
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="2:4">
+      <c r="B17" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2363,784 +2363,784 @@
       <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="F15" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="5" t="s">
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" spans="2:6">
+      <c r="B17" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="5" t="s">
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="F18" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="2:6">
+      <c r="B19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="5" t="s">
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="5" t="s">
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="2:6">
+      <c r="B22" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="5"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="5" t="s">
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="B23" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="5" t="s">
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="B24" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="5" t="s">
+      <c r="F24" s="5"/>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="B25" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="F25" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="2:6">
+      <c r="B26" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="C26" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="5" t="s">
+      <c r="F26" s="5"/>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="B27" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="5" t="s">
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28" spans="2:6">
+      <c r="B28" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="F28" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="2:6">
+      <c r="B29" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="5" t="s">
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="B30" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E30" s="5"/>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="5" t="s">
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="2:6">
+      <c r="B31" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="E31" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="F31" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="5" t="s">
+    <row r="32" spans="2:6">
+      <c r="B32" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E32" s="5"/>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="5" t="s">
+      <c r="F32" s="5"/>
+    </row>
+    <row r="33" spans="2:6">
+      <c r="B33" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="C33" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="E33" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="5"/>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="5" t="s">
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34" spans="2:6">
+      <c r="B34" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E34" s="5"/>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="5" t="s">
+      <c r="F34" s="5"/>
+    </row>
+    <row r="35" spans="2:6">
+      <c r="B35" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="F35" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
-      <c r="A36" s="5" t="s">
+    <row r="36" spans="2:6">
+      <c r="B36" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="D36" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E36" s="5"/>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" s="5" t="s">
+      <c r="F36" s="5"/>
+    </row>
+    <row r="37" spans="2:6">
+      <c r="B37" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="5"/>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" s="5" t="s">
+      <c r="F37" s="5"/>
+    </row>
+    <row r="38" spans="2:6">
+      <c r="B38" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="D38" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="F38" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
-      <c r="A39" s="5" t="s">
+    <row r="39" spans="2:6">
+      <c r="B39" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="C39" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E39" s="5"/>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" s="5" t="s">
+      <c r="F39" s="5"/>
+    </row>
+    <row r="40" spans="2:6">
+      <c r="B40" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E40" s="5"/>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" s="5" t="s">
+      <c r="F40" s="5"/>
+    </row>
+    <row r="41" spans="2:6">
+      <c r="B41" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="F41" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
-      <c r="A42" s="5" t="s">
+    <row r="42" spans="2:6">
+      <c r="B42" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E42" s="5"/>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" s="5" t="s">
+      <c r="F42" s="5"/>
+    </row>
+    <row r="43" spans="2:6">
+      <c r="B43" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="C43" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="D43" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E43" s="5"/>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" s="5" t="s">
+      <c r="F43" s="5"/>
+    </row>
+    <row r="44" spans="2:6">
+      <c r="B44" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="C44" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="D44" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="E44" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" s="5" t="s">
+      <c r="F44" s="5"/>
+    </row>
+    <row r="45" spans="2:6">
+      <c r="B45" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="C45" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="D45" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="E45" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="F45" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
-      <c r="A46" s="5" t="s">
+    <row r="46" spans="2:6">
+      <c r="B46" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="E46" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E46" s="5"/>
-    </row>
-    <row r="47" spans="1:5">
-      <c r="A47" s="5" t="s">
+      <c r="F46" s="5"/>
+    </row>
+    <row r="47" spans="2:6">
+      <c r="B47" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="C47" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="D47" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="E47" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E47" s="5"/>
-    </row>
-    <row r="48" spans="1:5">
-      <c r="A48" s="5" t="s">
+      <c r="F47" s="5"/>
+    </row>
+    <row r="48" spans="2:6">
+      <c r="B48" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="C48" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="D48" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="E48" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="F48" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
-      <c r="A49" s="5" t="s">
+    <row r="49" spans="2:6">
+      <c r="B49" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="C49" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="D49" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D49" s="5" t="s">
+      <c r="E49" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E49" s="5"/>
-    </row>
-    <row r="50" spans="1:5">
-      <c r="A50" s="5" t="s">
+      <c r="F49" s="5"/>
+    </row>
+    <row r="50" spans="2:6">
+      <c r="B50" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="C50" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="D50" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="E50" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E50" s="5"/>
-    </row>
-    <row r="51" spans="1:5">
-      <c r="A51" s="5" t="s">
+      <c r="F50" s="5"/>
+    </row>
+    <row r="51" spans="2:6">
+      <c r="B51" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="C51" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="D51" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="E51" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="F51" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
-      <c r="A52" s="5" t="s">
+    <row r="52" spans="2:6">
+      <c r="B52" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="C52" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="D52" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="E52" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E52" s="5"/>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="A53" s="5" t="s">
+      <c r="F52" s="5"/>
+    </row>
+    <row r="53" spans="2:6">
+      <c r="B53" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="C53" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="D53" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="E53" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E53" s="5"/>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" s="5" t="s">
+      <c r="F53" s="5"/>
+    </row>
+    <row r="54" spans="2:6">
+      <c r="B54" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="C54" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="D54" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="E54" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E54" s="5"/>
-    </row>
-    <row r="55" spans="1:5">
-      <c r="A55" s="5" t="s">
+      <c r="F54" s="5"/>
+    </row>
+    <row r="55" spans="2:6">
+      <c r="B55" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="C55" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="D55" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="5" t="s">
+      <c r="E55" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E55" s="5" t="s">
+      <c r="F55" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
-      <c r="A56" s="5" t="s">
+    <row r="56" spans="2:6">
+      <c r="B56" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="C56" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="D56" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D56" s="5" t="s">
+      <c r="E56" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E56" s="5"/>
-    </row>
-    <row r="57" spans="1:5">
-      <c r="A57" s="5" t="s">
+      <c r="F56" s="5"/>
+    </row>
+    <row r="57" spans="2:6">
+      <c r="B57" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="C57" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="D57" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="D57" s="5" t="s">
+      <c r="E57" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E57" s="5"/>
-    </row>
-    <row r="58" spans="1:5">
-      <c r="A58" s="5" t="s">
+      <c r="F57" s="5"/>
+    </row>
+    <row r="58" spans="2:6">
+      <c r="B58" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="C58" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="D58" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D58" s="5" t="s">
+      <c r="E58" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E58" s="5" t="s">
+      <c r="F58" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
-      <c r="A59" s="5" t="s">
+    <row r="59" spans="2:6">
+      <c r="B59" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="C59" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="D59" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="E59" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E59" s="5"/>
-    </row>
-    <row r="60" spans="1:5">
-      <c r="A60" s="5" t="s">
+      <c r="F59" s="5"/>
+    </row>
+    <row r="60" spans="2:6">
+      <c r="B60" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="C60" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="D60" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="E60" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E60" s="5"/>
-    </row>
-    <row r="61" spans="1:5">
-      <c r="A61" s="5" t="s">
+      <c r="F60" s="5"/>
+    </row>
+    <row r="61" spans="2:6">
+      <c r="B61" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="C61" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="D61" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="E61" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="F61" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
-      <c r="A62" s="5" t="s">
+    <row r="62" spans="2:6">
+      <c r="B62" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="C62" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="D62" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="E62" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3278,332 +3278,332 @@
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="2:4">
+      <c r="B17" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="2:4">
+      <c r="B18" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="2:4">
+      <c r="B19" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="2:4">
+      <c r="B20" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="2:4">
+      <c r="B21" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="2:4">
+      <c r="B22" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="2:4">
+      <c r="B23" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="5" t="s">
+    <row r="24" spans="2:4">
+      <c r="B24" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="2:4">
+      <c r="B25" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="2:4">
+      <c r="B26" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="C26" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="2:4">
+      <c r="B27" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="5" t="s">
+    <row r="28" spans="2:4">
+      <c r="B28" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="2:4">
+      <c r="B29" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="5" t="s">
+    <row r="30" spans="2:4">
+      <c r="B30" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="5" t="s">
+    <row r="31" spans="2:4">
+      <c r="B31" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="5" t="s">
+    <row r="32" spans="2:4">
+      <c r="B32" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="5" t="s">
+    <row r="33" spans="2:4">
+      <c r="B33" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="C33" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="5" t="s">
+    <row r="34" spans="2:4">
+      <c r="B34" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="5" t="s">
+    <row r="35" spans="2:4">
+      <c r="B35" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="5" t="s">
+    <row r="36" spans="2:4">
+      <c r="B36" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="D36" s="5" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="5" t="s">
+    <row r="37" spans="2:4">
+      <c r="B37" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="5" t="s">
+    <row r="38" spans="2:4">
+      <c r="B38" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="D38" s="5" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="5" t="s">
+    <row r="39" spans="2:4">
+      <c r="B39" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="C39" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="5" t="s">
+    <row r="40" spans="2:4">
+      <c r="B40" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="5" t="s">
+    <row r="41" spans="2:4">
+      <c r="B41" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
-      <c r="A42" s="5" t="s">
+    <row r="42" spans="2:4">
+      <c r="B42" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>194</v>
       </c>
     </row>
@@ -3743,35 +3743,35 @@
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>206</v>
       </c>
     </row>
@@ -3925,842 +3925,842 @@
       <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="2:5">
+      <c r="B18" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="2:5">
+      <c r="B19" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="2:5">
+      <c r="B20" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="2:5">
+      <c r="B21" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="2:5">
+      <c r="B22" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="2:5">
+      <c r="B23" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="5" t="s">
+    <row r="24" spans="2:5">
+      <c r="B24" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="2:5">
+      <c r="B25" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="2:5">
+      <c r="B26" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="C26" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="2:5">
+      <c r="B27" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="5" t="s">
+    <row r="28" spans="2:5">
+      <c r="B28" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="2:5">
+      <c r="B29" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="5" t="s">
+    <row r="30" spans="2:5">
+      <c r="B30" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="5" t="s">
+    <row r="31" spans="2:5">
+      <c r="B31" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="E31" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="5" t="s">
+    <row r="32" spans="2:5">
+      <c r="B32" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="5" t="s">
+    <row r="33" spans="2:5">
+      <c r="B33" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="C33" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="E33" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="5" t="s">
+    <row r="34" spans="2:5">
+      <c r="B34" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="5" t="s">
+    <row r="35" spans="2:5">
+      <c r="B35" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="5" t="s">
+    <row r="36" spans="2:5">
+      <c r="B36" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="D36" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="5" t="s">
+    <row r="37" spans="2:5">
+      <c r="B37" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="5" t="s">
+    <row r="38" spans="2:5">
+      <c r="B38" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="D38" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="5" t="s">
+    <row r="39" spans="2:5">
+      <c r="B39" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="C39" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="5" t="s">
+    <row r="40" spans="2:5">
+      <c r="B40" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="5" t="s">
+    <row r="41" spans="2:5">
+      <c r="B41" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="5" t="s">
+    <row r="42" spans="2:5">
+      <c r="B42" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="5" t="s">
+    <row r="43" spans="2:5">
+      <c r="B43" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="C43" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="D43" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="5" t="s">
+    <row r="44" spans="2:5">
+      <c r="B44" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="C44" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="D44" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="E44" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
-      <c r="A45" s="5" t="s">
+    <row r="45" spans="2:5">
+      <c r="B45" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="C45" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="D45" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="E45" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
-      <c r="A46" s="5" t="s">
+    <row r="46" spans="2:5">
+      <c r="B46" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="E46" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
-      <c r="A47" s="5" t="s">
+    <row r="47" spans="2:5">
+      <c r="B47" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="C47" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="D47" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="E47" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
-      <c r="A48" s="5" t="s">
+    <row r="48" spans="2:5">
+      <c r="B48" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="C48" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="D48" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="E48" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
-      <c r="A49" s="5" t="s">
+    <row r="49" spans="2:5">
+      <c r="B49" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="C49" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="D49" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D49" s="5" t="s">
+      <c r="E49" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
-      <c r="A50" s="5" t="s">
+    <row r="50" spans="2:5">
+      <c r="B50" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="C50" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="D50" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="E50" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
-      <c r="A51" s="5" t="s">
+    <row r="51" spans="2:5">
+      <c r="B51" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="C51" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="D51" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="E51" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
-      <c r="A52" s="5" t="s">
+    <row r="52" spans="2:5">
+      <c r="B52" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="C52" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="D52" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="E52" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
-      <c r="A53" s="5" t="s">
+    <row r="53" spans="2:5">
+      <c r="B53" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="C53" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="D53" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="E53" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
-      <c r="A54" s="5" t="s">
+    <row r="54" spans="2:5">
+      <c r="B54" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="C54" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="D54" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="E54" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
-      <c r="A55" s="5" t="s">
+    <row r="55" spans="2:5">
+      <c r="B55" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="C55" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="D55" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D55" s="5" t="s">
+      <c r="E55" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
-      <c r="A56" s="5" t="s">
+    <row r="56" spans="2:5">
+      <c r="B56" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="C56" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="D56" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D56" s="5" t="s">
+      <c r="E56" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
-      <c r="A57" s="5" t="s">
+    <row r="57" spans="2:5">
+      <c r="B57" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="C57" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="D57" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D57" s="5" t="s">
+      <c r="E57" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
-      <c r="A58" s="5" t="s">
+    <row r="58" spans="2:5">
+      <c r="B58" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="C58" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="D58" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D58" s="5" t="s">
+      <c r="E58" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
-      <c r="A59" s="5" t="s">
+    <row r="59" spans="2:5">
+      <c r="B59" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="C59" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="D59" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="E59" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
-      <c r="A60" s="5" t="s">
+    <row r="60" spans="2:5">
+      <c r="B60" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="C60" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="D60" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="E60" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
-      <c r="A61" s="5" t="s">
+    <row r="61" spans="2:5">
+      <c r="B61" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="C61" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="D61" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="E61" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
-      <c r="A62" s="5" t="s">
+    <row r="62" spans="2:5">
+      <c r="B62" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="C62" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="D62" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="E62" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
-      <c r="A63" s="5" t="s">
+    <row r="63" spans="2:5">
+      <c r="B63" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="C63" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="D63" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="E63" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
-      <c r="A64" s="5" t="s">
+    <row r="64" spans="2:5">
+      <c r="B64" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="C64" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="C64" s="5" t="s">
+      <c r="D64" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D64" s="5" t="s">
+      <c r="E64" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
-      <c r="A65" s="5" t="s">
+    <row r="65" spans="2:5">
+      <c r="B65" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="C65" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="D65" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D65" s="5" t="s">
+      <c r="E65" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
-      <c r="A66" s="5" t="s">
+    <row r="66" spans="2:5">
+      <c r="B66" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="C66" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="D66" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="E66" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
-      <c r="A67" s="5" t="s">
+    <row r="67" spans="2:5">
+      <c r="B67" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="C67" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="C67" s="5" t="s">
+      <c r="D67" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D67" s="5" t="s">
+      <c r="E67" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
-      <c r="A68" s="5" t="s">
+    <row r="68" spans="2:5">
+      <c r="B68" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="C68" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="C68" s="5" t="s">
+      <c r="D68" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D68" s="5" t="s">
+      <c r="E68" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
-      <c r="A69" s="5" t="s">
+    <row r="69" spans="2:5">
+      <c r="B69" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="C69" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="D69" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D69" s="5" t="s">
+      <c r="E69" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="70" spans="1:4">
-      <c r="A70" s="5" t="s">
+    <row r="70" spans="2:5">
+      <c r="B70" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="C70" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="C70" s="5" t="s">
+      <c r="D70" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="E70" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
-      <c r="A71" s="5" t="s">
+    <row r="71" spans="2:5">
+      <c r="B71" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="C71" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="C71" s="5" t="s">
+      <c r="D71" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D71" s="5" t="s">
+      <c r="E71" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:4">
-      <c r="A72" s="5" t="s">
+    <row r="72" spans="2:5">
+      <c r="B72" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="C72" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="C72" s="5" t="s">
+      <c r="D72" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D72" s="5" t="s">
+      <c r="E72" s="5" t="s">
         <v>49</v>
       </c>
     </row>
@@ -4921,142 +4921,142 @@
       <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="2:5">
+      <c r="B18" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="2:5">
+      <c r="B19" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="2:5">
+      <c r="B20" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="2:5">
+      <c r="B21" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="2:5">
+      <c r="B22" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>305</v>
       </c>
     </row>
@@ -5211,422 +5211,422 @@
       <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>321</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="2:5">
+      <c r="B18" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="2:5">
+      <c r="B19" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="2:5">
+      <c r="B20" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="2:5">
+      <c r="B21" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="2:5">
+      <c r="B22" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="2:5">
+      <c r="B23" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="5" t="s">
+    <row r="24" spans="2:5">
+      <c r="B24" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="2:5">
+      <c r="B25" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="2:5">
+      <c r="B26" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="C26" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="2:5">
+      <c r="B27" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="5" t="s">
+    <row r="28" spans="2:5">
+      <c r="B28" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="2:5">
+      <c r="B29" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="5" t="s">
+    <row r="30" spans="2:5">
+      <c r="B30" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>381</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>382</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="5" t="s">
+    <row r="31" spans="2:5">
+      <c r="B31" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>386</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="E31" s="5" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="5" t="s">
+    <row r="32" spans="2:5">
+      <c r="B32" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="5" t="s">
+    <row r="33" spans="2:5">
+      <c r="B33" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="C33" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="E33" s="5" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="5" t="s">
+    <row r="34" spans="2:5">
+      <c r="B34" s="5" t="s">
         <v>396</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>397</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>398</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="5" t="s">
+    <row r="35" spans="2:5">
+      <c r="B35" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>401</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="5" t="s">
+    <row r="36" spans="2:5">
+      <c r="B36" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="D36" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="5" t="s">
+    <row r="37" spans="2:5">
+      <c r="B37" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="5" t="s">
+    <row r="38" spans="2:5">
+      <c r="B38" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>413</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="D38" s="5" t="s">
         <v>414</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="5" t="s">
+    <row r="39" spans="2:5">
+      <c r="B39" s="5" t="s">
         <v>416</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="C39" s="5" t="s">
         <v>417</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="5" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="5" t="s">
+    <row r="40" spans="2:5">
+      <c r="B40" s="5" t="s">
         <v>420</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>422</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="5" t="s">
+    <row r="41" spans="2:5">
+      <c r="B41" s="5" t="s">
         <v>424</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="5" t="s">
+    <row r="42" spans="2:5">
+      <c r="B42" s="5" t="s">
         <v>428</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>429</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>431</v>
       </c>
     </row>
@@ -5767,112 +5767,112 @@
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>439</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>441</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>442</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>443</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="2:4">
+      <c r="B17" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>445</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="2:4">
+      <c r="B18" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>447</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="2:4">
+      <c r="B19" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>449</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="2:4">
+      <c r="B20" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="2:4">
+      <c r="B21" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>453</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="2:4">
+      <c r="B22" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>455</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>456</v>
       </c>
     </row>

</xml_diff>